<commit_message>
feat: enhance attendance tracking and parent registration flow with new functions and improved data handling
</commit_message>
<xml_diff>
--- a/assets/admin/attendance/templates/SF4_Blank_SHS.xlsx
+++ b/assets/admin/attendance/templates/SF4_Blank_SHS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\L4T\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\L4T\Documents\Website\ulhs.github.io\assets\admin\attendance\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398699E5-0CDF-42CF-80C2-B4BB345AD180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE550BFF-F59E-429C-AB5B-989372F8BFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="month" sheetId="2" r:id="rId1"/>
@@ -264,7 +264,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="56">
+  <borders count="57">
     <border>
       <left/>
       <right/>
@@ -955,11 +955,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1185,30 +1200,76 @@
     <xf numFmtId="2" fontId="15" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1216,8 +1277,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1225,10 +1289,13 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1242,56 +1309,35 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1581,7 +1627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:BD227"/>
+  <dimension ref="A1:BD228"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.08984375" customWidth="1"/>
@@ -1601,237 +1647,237 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82"/>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
-      <c r="Q1" s="82"/>
-      <c r="R1" s="82"/>
-      <c r="S1" s="82"/>
-      <c r="T1" s="82"/>
-      <c r="U1" s="82"/>
-      <c r="V1" s="82"/>
-      <c r="W1" s="82"/>
-      <c r="X1" s="82"/>
-      <c r="Y1" s="82"/>
-      <c r="Z1" s="82"/>
-      <c r="AA1" s="82"/>
-      <c r="AB1" s="82"/>
-      <c r="AC1" s="82"/>
-      <c r="AD1" s="82"/>
-      <c r="AE1" s="82"/>
-      <c r="AF1" s="82"/>
-      <c r="AG1" s="82"/>
-      <c r="AH1" s="82"/>
-      <c r="AI1" s="82"/>
-      <c r="AJ1" s="82"/>
-      <c r="AK1" s="82"/>
-      <c r="AL1" s="82"/>
-      <c r="AM1" s="82"/>
-      <c r="AN1" s="82"/>
-      <c r="AO1" s="82"/>
-      <c r="AP1" s="82"/>
-      <c r="AQ1" s="82"/>
-      <c r="AR1" s="82"/>
-      <c r="AS1" s="82"/>
-      <c r="AT1" s="82"/>
-      <c r="AU1" s="82"/>
-      <c r="AV1" s="82"/>
-      <c r="AW1" s="82"/>
-      <c r="AX1" s="82"/>
-      <c r="AY1" s="82"/>
-      <c r="AZ1" s="82"/>
-      <c r="BA1" s="82"/>
-      <c r="BB1" s="82"/>
-      <c r="BC1" s="82"/>
-      <c r="BD1" s="82"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
+      <c r="L1" s="87"/>
+      <c r="M1" s="87"/>
+      <c r="N1" s="87"/>
+      <c r="O1" s="87"/>
+      <c r="P1" s="87"/>
+      <c r="Q1" s="87"/>
+      <c r="R1" s="87"/>
+      <c r="S1" s="87"/>
+      <c r="T1" s="87"/>
+      <c r="U1" s="87"/>
+      <c r="V1" s="87"/>
+      <c r="W1" s="87"/>
+      <c r="X1" s="87"/>
+      <c r="Y1" s="87"/>
+      <c r="Z1" s="87"/>
+      <c r="AA1" s="87"/>
+      <c r="AB1" s="87"/>
+      <c r="AC1" s="87"/>
+      <c r="AD1" s="87"/>
+      <c r="AE1" s="87"/>
+      <c r="AF1" s="87"/>
+      <c r="AG1" s="87"/>
+      <c r="AH1" s="87"/>
+      <c r="AI1" s="87"/>
+      <c r="AJ1" s="87"/>
+      <c r="AK1" s="87"/>
+      <c r="AL1" s="87"/>
+      <c r="AM1" s="87"/>
+      <c r="AN1" s="87"/>
+      <c r="AO1" s="87"/>
+      <c r="AP1" s="87"/>
+      <c r="AQ1" s="87"/>
+      <c r="AR1" s="87"/>
+      <c r="AS1" s="87"/>
+      <c r="AT1" s="87"/>
+      <c r="AU1" s="87"/>
+      <c r="AV1" s="87"/>
+      <c r="AW1" s="87"/>
+      <c r="AX1" s="87"/>
+      <c r="AY1" s="87"/>
+      <c r="AZ1" s="87"/>
+      <c r="BA1" s="87"/>
+      <c r="BB1" s="87"/>
+      <c r="BC1" s="87"/>
+      <c r="BD1" s="87"/>
     </row>
     <row r="2" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A2" s="82"/>
-      <c r="B2" s="82"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="82"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="82"/>
-      <c r="Q2" s="82"/>
-      <c r="R2" s="82"/>
-      <c r="S2" s="82"/>
-      <c r="T2" s="82"/>
-      <c r="U2" s="82"/>
-      <c r="V2" s="82"/>
-      <c r="W2" s="82"/>
-      <c r="X2" s="82"/>
-      <c r="Y2" s="82"/>
-      <c r="Z2" s="82"/>
-      <c r="AA2" s="82"/>
-      <c r="AB2" s="82"/>
-      <c r="AC2" s="82"/>
-      <c r="AD2" s="82"/>
-      <c r="AE2" s="82"/>
-      <c r="AF2" s="82"/>
-      <c r="AG2" s="82"/>
-      <c r="AH2" s="82"/>
-      <c r="AI2" s="82"/>
-      <c r="AJ2" s="82"/>
-      <c r="AK2" s="82"/>
-      <c r="AL2" s="82"/>
-      <c r="AM2" s="82"/>
-      <c r="AN2" s="82"/>
-      <c r="AO2" s="82"/>
-      <c r="AP2" s="82"/>
-      <c r="AQ2" s="82"/>
-      <c r="AR2" s="82"/>
-      <c r="AS2" s="82"/>
-      <c r="AT2" s="82"/>
-      <c r="AU2" s="82"/>
-      <c r="AV2" s="82"/>
-      <c r="AW2" s="82"/>
-      <c r="AX2" s="82"/>
-      <c r="AY2" s="82"/>
-      <c r="AZ2" s="82"/>
-      <c r="BA2" s="82"/>
-      <c r="BB2" s="82"/>
-      <c r="BC2" s="82"/>
-      <c r="BD2" s="82"/>
+      <c r="A2" s="87"/>
+      <c r="B2" s="87"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="87"/>
+      <c r="L2" s="87"/>
+      <c r="M2" s="87"/>
+      <c r="N2" s="87"/>
+      <c r="O2" s="87"/>
+      <c r="P2" s="87"/>
+      <c r="Q2" s="87"/>
+      <c r="R2" s="87"/>
+      <c r="S2" s="87"/>
+      <c r="T2" s="87"/>
+      <c r="U2" s="87"/>
+      <c r="V2" s="87"/>
+      <c r="W2" s="87"/>
+      <c r="X2" s="87"/>
+      <c r="Y2" s="87"/>
+      <c r="Z2" s="87"/>
+      <c r="AA2" s="87"/>
+      <c r="AB2" s="87"/>
+      <c r="AC2" s="87"/>
+      <c r="AD2" s="87"/>
+      <c r="AE2" s="87"/>
+      <c r="AF2" s="87"/>
+      <c r="AG2" s="87"/>
+      <c r="AH2" s="87"/>
+      <c r="AI2" s="87"/>
+      <c r="AJ2" s="87"/>
+      <c r="AK2" s="87"/>
+      <c r="AL2" s="87"/>
+      <c r="AM2" s="87"/>
+      <c r="AN2" s="87"/>
+      <c r="AO2" s="87"/>
+      <c r="AP2" s="87"/>
+      <c r="AQ2" s="87"/>
+      <c r="AR2" s="87"/>
+      <c r="AS2" s="87"/>
+      <c r="AT2" s="87"/>
+      <c r="AU2" s="87"/>
+      <c r="AV2" s="87"/>
+      <c r="AW2" s="87"/>
+      <c r="AX2" s="87"/>
+      <c r="AY2" s="87"/>
+      <c r="AZ2" s="87"/>
+      <c r="BA2" s="87"/>
+      <c r="BB2" s="87"/>
+      <c r="BC2" s="87"/>
+      <c r="BD2" s="87"/>
     </row>
     <row r="3" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A3" s="83"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="82"/>
-      <c r="L3" s="82"/>
-      <c r="M3" s="82"/>
-      <c r="N3" s="82"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="82"/>
-      <c r="R3" s="82"/>
-      <c r="S3" s="82"/>
-      <c r="T3" s="82"/>
-      <c r="U3" s="82"/>
-      <c r="V3" s="82"/>
-      <c r="W3" s="82"/>
-      <c r="X3" s="82"/>
-      <c r="Y3" s="82"/>
-      <c r="Z3" s="82"/>
-      <c r="AA3" s="82"/>
-      <c r="AB3" s="82"/>
-      <c r="AC3" s="82"/>
-      <c r="AD3" s="82"/>
-      <c r="AE3" s="82"/>
-      <c r="AF3" s="82"/>
-      <c r="AG3" s="82"/>
-      <c r="AH3" s="82"/>
-      <c r="AI3" s="82"/>
-      <c r="AJ3" s="82"/>
-      <c r="AK3" s="82"/>
-      <c r="AL3" s="82"/>
-      <c r="AM3" s="82"/>
-      <c r="AN3" s="82"/>
-      <c r="AO3" s="82"/>
-      <c r="AP3" s="82"/>
-      <c r="AQ3" s="82"/>
-      <c r="AR3" s="82"/>
-      <c r="AS3" s="82"/>
-      <c r="AT3" s="82"/>
-      <c r="AU3" s="82"/>
-      <c r="AV3" s="82"/>
-      <c r="AW3" s="82"/>
-      <c r="AX3" s="82"/>
-      <c r="AY3" s="82"/>
-      <c r="AZ3" s="82"/>
-      <c r="BA3" s="82"/>
-      <c r="BB3" s="82"/>
-      <c r="BC3" s="82"/>
-      <c r="BD3" s="82"/>
+      <c r="A3" s="90"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="87"/>
+      <c r="L3" s="87"/>
+      <c r="M3" s="87"/>
+      <c r="N3" s="87"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="87"/>
+      <c r="Q3" s="87"/>
+      <c r="R3" s="87"/>
+      <c r="S3" s="87"/>
+      <c r="T3" s="87"/>
+      <c r="U3" s="87"/>
+      <c r="V3" s="87"/>
+      <c r="W3" s="87"/>
+      <c r="X3" s="87"/>
+      <c r="Y3" s="87"/>
+      <c r="Z3" s="87"/>
+      <c r="AA3" s="87"/>
+      <c r="AB3" s="87"/>
+      <c r="AC3" s="87"/>
+      <c r="AD3" s="87"/>
+      <c r="AE3" s="87"/>
+      <c r="AF3" s="87"/>
+      <c r="AG3" s="87"/>
+      <c r="AH3" s="87"/>
+      <c r="AI3" s="87"/>
+      <c r="AJ3" s="87"/>
+      <c r="AK3" s="87"/>
+      <c r="AL3" s="87"/>
+      <c r="AM3" s="87"/>
+      <c r="AN3" s="87"/>
+      <c r="AO3" s="87"/>
+      <c r="AP3" s="87"/>
+      <c r="AQ3" s="87"/>
+      <c r="AR3" s="87"/>
+      <c r="AS3" s="87"/>
+      <c r="AT3" s="87"/>
+      <c r="AU3" s="87"/>
+      <c r="AV3" s="87"/>
+      <c r="AW3" s="87"/>
+      <c r="AX3" s="87"/>
+      <c r="AY3" s="87"/>
+      <c r="AZ3" s="87"/>
+      <c r="BA3" s="87"/>
+      <c r="BB3" s="87"/>
+      <c r="BC3" s="87"/>
+      <c r="BD3" s="87"/>
     </row>
     <row r="4" spans="1:56" ht="16.5" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="80"/>
-      <c r="K4" s="80"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="113" t="s">
+      <c r="C4" s="85"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="82"/>
+      <c r="M4" s="108" t="s">
         <v>3</v>
       </c>
-      <c r="N4" s="82"/>
-      <c r="O4" s="84"/>
-      <c r="P4" s="79"/>
-      <c r="Q4" s="80"/>
-      <c r="R4" s="80"/>
-      <c r="S4" s="80"/>
-      <c r="T4" s="80"/>
-      <c r="U4" s="80"/>
-      <c r="V4" s="80"/>
-      <c r="W4" s="80"/>
-      <c r="X4" s="81"/>
-      <c r="Y4" s="110" t="s">
+      <c r="N4" s="87"/>
+      <c r="O4" s="88"/>
+      <c r="P4" s="85"/>
+      <c r="Q4" s="81"/>
+      <c r="R4" s="81"/>
+      <c r="S4" s="81"/>
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="82"/>
+      <c r="Y4" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="Z4" s="82"/>
-      <c r="AA4" s="82"/>
-      <c r="AB4" s="84"/>
-      <c r="AC4" s="79"/>
-      <c r="AD4" s="80"/>
-      <c r="AE4" s="80"/>
-      <c r="AF4" s="80"/>
-      <c r="AG4" s="80"/>
-      <c r="AH4" s="80"/>
-      <c r="AI4" s="80"/>
-      <c r="AJ4" s="80"/>
-      <c r="AK4" s="80"/>
-      <c r="AL4" s="80"/>
-      <c r="AM4" s="80"/>
-      <c r="AN4" s="80"/>
-      <c r="AO4" s="81"/>
-      <c r="AP4" s="110" t="s">
+      <c r="Z4" s="87"/>
+      <c r="AA4" s="87"/>
+      <c r="AB4" s="88"/>
+      <c r="AC4" s="85"/>
+      <c r="AD4" s="81"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="81"/>
+      <c r="AG4" s="81"/>
+      <c r="AH4" s="81"/>
+      <c r="AI4" s="81"/>
+      <c r="AJ4" s="81"/>
+      <c r="AK4" s="81"/>
+      <c r="AL4" s="81"/>
+      <c r="AM4" s="81"/>
+      <c r="AN4" s="81"/>
+      <c r="AO4" s="82"/>
+      <c r="AP4" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="AQ4" s="82"/>
-      <c r="AR4" s="84"/>
-      <c r="AS4" s="79"/>
-      <c r="AT4" s="80"/>
-      <c r="AU4" s="81"/>
+      <c r="AQ4" s="87"/>
+      <c r="AR4" s="88"/>
+      <c r="AS4" s="85"/>
+      <c r="AT4" s="81"/>
+      <c r="AU4" s="82"/>
       <c r="AV4" s="2"/>
       <c r="AW4" s="2"/>
       <c r="AX4" s="2"/>
@@ -1905,66 +1951,66 @@
       <c r="B6" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="96"/>
-      <c r="D6" s="80"/>
-      <c r="E6" s="80"/>
-      <c r="F6" s="80"/>
-      <c r="G6" s="81"/>
+      <c r="C6" s="91"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="81"/>
+      <c r="F6" s="81"/>
+      <c r="G6" s="82"/>
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
       <c r="J6" s="3"/>
-      <c r="K6" s="110" t="s">
+      <c r="K6" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="82"/>
-      <c r="M6" s="82"/>
-      <c r="N6" s="82"/>
-      <c r="O6" s="84"/>
-      <c r="P6" s="96"/>
-      <c r="Q6" s="80"/>
-      <c r="R6" s="80"/>
-      <c r="S6" s="80"/>
-      <c r="T6" s="80"/>
-      <c r="U6" s="81"/>
+      <c r="L6" s="87"/>
+      <c r="M6" s="87"/>
+      <c r="N6" s="87"/>
+      <c r="O6" s="88"/>
+      <c r="P6" s="91"/>
+      <c r="Q6" s="81"/>
+      <c r="R6" s="81"/>
+      <c r="S6" s="81"/>
+      <c r="T6" s="81"/>
+      <c r="U6" s="82"/>
       <c r="V6" s="23"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
-      <c r="Y6" s="110" t="s">
+      <c r="Y6" s="86" t="s">
         <v>5</v>
       </c>
-      <c r="Z6" s="82"/>
-      <c r="AA6" s="82"/>
-      <c r="AB6" s="82"/>
-      <c r="AC6" s="82"/>
-      <c r="AD6" s="82"/>
-      <c r="AE6" s="84"/>
-      <c r="AF6" s="96"/>
-      <c r="AG6" s="80"/>
-      <c r="AH6" s="80"/>
-      <c r="AI6" s="80"/>
-      <c r="AJ6" s="80"/>
-      <c r="AK6" s="80"/>
-      <c r="AL6" s="80"/>
-      <c r="AM6" s="80"/>
-      <c r="AN6" s="80"/>
-      <c r="AO6" s="81"/>
+      <c r="Z6" s="87"/>
+      <c r="AA6" s="87"/>
+      <c r="AB6" s="87"/>
+      <c r="AC6" s="87"/>
+      <c r="AD6" s="87"/>
+      <c r="AE6" s="88"/>
+      <c r="AF6" s="91"/>
+      <c r="AG6" s="81"/>
+      <c r="AH6" s="81"/>
+      <c r="AI6" s="81"/>
+      <c r="AJ6" s="81"/>
+      <c r="AK6" s="81"/>
+      <c r="AL6" s="81"/>
+      <c r="AM6" s="81"/>
+      <c r="AN6" s="81"/>
+      <c r="AO6" s="82"/>
       <c r="AP6" s="2"/>
-      <c r="AQ6" s="104" t="s">
+      <c r="AQ6" s="124" t="s">
         <v>24</v>
       </c>
-      <c r="AR6" s="82"/>
-      <c r="AS6" s="82"/>
-      <c r="AT6" s="82"/>
-      <c r="AU6" s="82"/>
-      <c r="AV6" s="84"/>
-      <c r="AW6" s="105"/>
-      <c r="AX6" s="80"/>
-      <c r="AY6" s="80"/>
-      <c r="AZ6" s="80"/>
-      <c r="BA6" s="80"/>
-      <c r="BB6" s="80"/>
-      <c r="BC6" s="80"/>
-      <c r="BD6" s="81"/>
+      <c r="AR6" s="87"/>
+      <c r="AS6" s="87"/>
+      <c r="AT6" s="87"/>
+      <c r="AU6" s="87"/>
+      <c r="AV6" s="88"/>
+      <c r="AW6" s="125"/>
+      <c r="AX6" s="81"/>
+      <c r="AY6" s="81"/>
+      <c r="AZ6" s="81"/>
+      <c r="BA6" s="81"/>
+      <c r="BB6" s="81"/>
+      <c r="BC6" s="81"/>
+      <c r="BD6" s="82"/>
     </row>
     <row r="7" spans="1:56" ht="16.5" customHeight="1">
       <c r="A7" s="5"/>
@@ -2083,176 +2129,176 @@
       <c r="BD8" s="1"/>
     </row>
     <row r="9" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A9" s="119" t="s">
+      <c r="A9" s="96" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="119" t="s">
+      <c r="B9" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="98" t="s">
+      <c r="C9" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="85"/>
-      <c r="E9" s="99"/>
-      <c r="F9" s="117" t="s">
+      <c r="D9" s="116"/>
+      <c r="E9" s="117"/>
+      <c r="F9" s="92" t="s">
         <v>7</v>
       </c>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
-      <c r="L9" s="115" t="s">
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="93"/>
+      <c r="J9" s="93"/>
+      <c r="K9" s="94"/>
+      <c r="L9" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="M9" s="88"/>
-      <c r="N9" s="88"/>
-      <c r="O9" s="88"/>
-      <c r="P9" s="88"/>
-      <c r="Q9" s="88"/>
-      <c r="R9" s="88"/>
-      <c r="S9" s="88"/>
-      <c r="T9" s="90"/>
-      <c r="U9" s="118" t="s">
+      <c r="M9" s="93"/>
+      <c r="N9" s="93"/>
+      <c r="O9" s="93"/>
+      <c r="P9" s="93"/>
+      <c r="Q9" s="93"/>
+      <c r="R9" s="93"/>
+      <c r="S9" s="93"/>
+      <c r="T9" s="102"/>
+      <c r="U9" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="V9" s="88"/>
-      <c r="W9" s="88"/>
-      <c r="X9" s="88"/>
-      <c r="Y9" s="88"/>
-      <c r="Z9" s="88"/>
-      <c r="AA9" s="88"/>
-      <c r="AB9" s="88"/>
-      <c r="AC9" s="89"/>
-      <c r="AD9" s="123" t="s">
+      <c r="V9" s="93"/>
+      <c r="W9" s="93"/>
+      <c r="X9" s="93"/>
+      <c r="Y9" s="93"/>
+      <c r="Z9" s="93"/>
+      <c r="AA9" s="93"/>
+      <c r="AB9" s="93"/>
+      <c r="AC9" s="94"/>
+      <c r="AD9" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="AE9" s="88"/>
-      <c r="AF9" s="88"/>
-      <c r="AG9" s="88"/>
-      <c r="AH9" s="88"/>
-      <c r="AI9" s="88"/>
-      <c r="AJ9" s="88"/>
-      <c r="AK9" s="88"/>
-      <c r="AL9" s="90"/>
-      <c r="AM9" s="117" t="s">
+      <c r="AE9" s="93"/>
+      <c r="AF9" s="93"/>
+      <c r="AG9" s="93"/>
+      <c r="AH9" s="93"/>
+      <c r="AI9" s="93"/>
+      <c r="AJ9" s="93"/>
+      <c r="AK9" s="93"/>
+      <c r="AL9" s="102"/>
+      <c r="AM9" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="AN9" s="88"/>
-      <c r="AO9" s="88"/>
-      <c r="AP9" s="88"/>
-      <c r="AQ9" s="88"/>
-      <c r="AR9" s="88"/>
-      <c r="AS9" s="88"/>
-      <c r="AT9" s="88"/>
-      <c r="AU9" s="89"/>
-      <c r="AV9" s="123" t="s">
+      <c r="AN9" s="93"/>
+      <c r="AO9" s="93"/>
+      <c r="AP9" s="93"/>
+      <c r="AQ9" s="93"/>
+      <c r="AR9" s="93"/>
+      <c r="AS9" s="93"/>
+      <c r="AT9" s="93"/>
+      <c r="AU9" s="94"/>
+      <c r="AV9" s="101" t="s">
         <v>28</v>
       </c>
-      <c r="AW9" s="88"/>
-      <c r="AX9" s="88"/>
-      <c r="AY9" s="88"/>
-      <c r="AZ9" s="88"/>
-      <c r="BA9" s="88"/>
-      <c r="BB9" s="88"/>
-      <c r="BC9" s="88"/>
-      <c r="BD9" s="89"/>
+      <c r="AW9" s="93"/>
+      <c r="AX9" s="93"/>
+      <c r="AY9" s="93"/>
+      <c r="AZ9" s="93"/>
+      <c r="BA9" s="93"/>
+      <c r="BB9" s="93"/>
+      <c r="BC9" s="93"/>
+      <c r="BD9" s="94"/>
     </row>
     <row r="10" spans="1:56" ht="21.75" customHeight="1">
-      <c r="A10" s="120"/>
-      <c r="B10" s="120"/>
-      <c r="C10" s="100"/>
-      <c r="D10" s="87"/>
-      <c r="E10" s="91"/>
-      <c r="F10" s="97" t="s">
+      <c r="A10" s="97"/>
+      <c r="B10" s="97"/>
+      <c r="C10" s="118"/>
+      <c r="D10" s="119"/>
+      <c r="E10" s="120"/>
+      <c r="F10" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="80"/>
-      <c r="H10" s="81"/>
-      <c r="I10" s="122" t="s">
+      <c r="G10" s="81"/>
+      <c r="H10" s="82"/>
+      <c r="I10" s="100" t="s">
         <v>29</v>
       </c>
-      <c r="J10" s="80"/>
-      <c r="K10" s="106"/>
-      <c r="L10" s="114" t="s">
+      <c r="J10" s="81"/>
+      <c r="K10" s="83"/>
+      <c r="L10" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="80"/>
-      <c r="N10" s="81"/>
-      <c r="O10" s="101" t="s">
+      <c r="M10" s="81"/>
+      <c r="N10" s="82"/>
+      <c r="O10" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="P10" s="80"/>
-      <c r="Q10" s="81"/>
-      <c r="R10" s="101" t="s">
+      <c r="P10" s="81"/>
+      <c r="Q10" s="82"/>
+      <c r="R10" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="S10" s="80"/>
-      <c r="T10" s="81"/>
-      <c r="U10" s="124" t="s">
+      <c r="S10" s="81"/>
+      <c r="T10" s="82"/>
+      <c r="U10" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="V10" s="80"/>
-      <c r="W10" s="81"/>
-      <c r="X10" s="101" t="s">
+      <c r="V10" s="81"/>
+      <c r="W10" s="82"/>
+      <c r="X10" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="Y10" s="80"/>
-      <c r="Z10" s="81"/>
-      <c r="AA10" s="101" t="s">
+      <c r="Y10" s="81"/>
+      <c r="Z10" s="82"/>
+      <c r="AA10" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="AB10" s="80"/>
-      <c r="AC10" s="106"/>
-      <c r="AD10" s="114" t="s">
+      <c r="AB10" s="81"/>
+      <c r="AC10" s="83"/>
+      <c r="AD10" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="AE10" s="80"/>
-      <c r="AF10" s="81"/>
-      <c r="AG10" s="101" t="s">
+      <c r="AE10" s="81"/>
+      <c r="AF10" s="82"/>
+      <c r="AG10" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="AH10" s="80"/>
-      <c r="AI10" s="81"/>
-      <c r="AJ10" s="101" t="s">
+      <c r="AH10" s="81"/>
+      <c r="AI10" s="82"/>
+      <c r="AJ10" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="AK10" s="80"/>
-      <c r="AL10" s="81"/>
-      <c r="AM10" s="124" t="s">
+      <c r="AK10" s="81"/>
+      <c r="AL10" s="82"/>
+      <c r="AM10" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="AN10" s="80"/>
-      <c r="AO10" s="81"/>
-      <c r="AP10" s="101" t="s">
+      <c r="AN10" s="81"/>
+      <c r="AO10" s="82"/>
+      <c r="AP10" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="AQ10" s="80"/>
-      <c r="AR10" s="81"/>
-      <c r="AS10" s="101" t="s">
+      <c r="AQ10" s="81"/>
+      <c r="AR10" s="82"/>
+      <c r="AS10" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="AT10" s="80"/>
-      <c r="AU10" s="106"/>
-      <c r="AV10" s="114" t="s">
+      <c r="AT10" s="81"/>
+      <c r="AU10" s="83"/>
+      <c r="AV10" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="AW10" s="80"/>
-      <c r="AX10" s="81"/>
-      <c r="AY10" s="101" t="s">
+      <c r="AW10" s="81"/>
+      <c r="AX10" s="82"/>
+      <c r="AY10" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="AZ10" s="80"/>
-      <c r="BA10" s="81"/>
-      <c r="BB10" s="101" t="s">
+      <c r="AZ10" s="81"/>
+      <c r="BA10" s="82"/>
+      <c r="BB10" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="BC10" s="80"/>
-      <c r="BD10" s="106"/>
+      <c r="BC10" s="81"/>
+      <c r="BD10" s="83"/>
     </row>
     <row r="11" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A11" s="121"/>
-      <c r="B11" s="121"/>
+      <c r="A11" s="98"/>
+      <c r="B11" s="98"/>
       <c r="C11" s="10" t="s">
         <v>12</v>
       </c>
@@ -2422,19 +2468,19 @@
       <c r="C12" s="27"/>
       <c r="D12" s="27"/>
       <c r="E12" s="28">
-        <f t="shared" ref="E12:E18" si="0">SUM(C12:D12)</f>
+        <f t="shared" ref="E12:E19" si="0">SUM(C12:D12)</f>
         <v>0</v>
       </c>
       <c r="F12" s="55"/>
       <c r="G12" s="56"/>
       <c r="H12" s="56">
-        <f t="shared" ref="H12:H18" si="1">SUM(F12:G12)</f>
+        <f t="shared" ref="H12:H19" si="1">SUM(F12:G12)</f>
         <v>0</v>
       </c>
       <c r="I12" s="56"/>
       <c r="J12" s="56"/>
       <c r="K12" s="57" t="e">
-        <f t="shared" ref="K12:K18" si="2">AVERAGE(I12:J12)</f>
+        <f t="shared" ref="K12:K19" si="2">AVERAGE(I12:J12)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="L12" s="52">
@@ -2731,10 +2777,10 @@
       </c>
     </row>
     <row r="14" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A14" s="111" t="s">
+      <c r="A14" s="106" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="112"/>
+      <c r="B14" s="107"/>
       <c r="C14" s="33">
         <f>SUM(C12:C13)</f>
         <v>0</v>
@@ -2907,18 +2953,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:56" ht="30" customHeight="1">
+    <row r="15" spans="1:56" ht="30" customHeight="1" thickBot="1">
       <c r="A15" s="35"/>
       <c r="B15" s="36"/>
       <c r="C15" s="37"/>
       <c r="D15" s="38"/>
-      <c r="E15" s="38">
+      <c r="E15" s="133">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F15" s="55"/>
       <c r="G15" s="56"/>
-      <c r="H15" s="56">
+      <c r="H15" s="62">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -3064,24 +3110,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:56" ht="30" customHeight="1">
-      <c r="A16" s="39"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42">
+    <row r="16" spans="1:56" s="79" customFormat="1" ht="30" customHeight="1">
+      <c r="A16" s="126"/>
+      <c r="B16" s="127"/>
+      <c r="C16" s="128"/>
+      <c r="D16" s="129"/>
+      <c r="E16" s="134">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F16" s="58"/>
-      <c r="G16" s="59"/>
-      <c r="H16" s="59">
+      <c r="F16" s="132"/>
+      <c r="G16" s="131"/>
+      <c r="H16" s="135">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I16" s="59"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="60" t="e">
+      <c r="I16" s="132"/>
+      <c r="J16" s="130"/>
+      <c r="K16" s="57" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
@@ -3221,44 +3267,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A17" s="107" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="108"/>
-      <c r="C17" s="43">
-        <f>SUM(C15:C16)</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="43">
-        <f>SUM(D15:D16)</f>
-        <v>0</v>
-      </c>
+    <row r="17" spans="1:56" ht="30" customHeight="1" thickBot="1">
+      <c r="A17" s="39"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
       <c r="E17" s="44">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F17" s="65">
-        <f>SUM(F15:F16)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="66">
-        <f>SUM(G15:G16)</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="66">
+      <c r="F17" s="58"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="130">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I17" s="66" t="e">
-        <f>AVERAGE(I15:I16)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J17" s="66" t="e">
-        <f>AVERAGE(J15:J16)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K17" s="67" t="e">
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="60" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
@@ -3399,419 +3425,538 @@
       </c>
     </row>
     <row r="18" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A18" s="109" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="108"/>
-      <c r="C18" s="45">
-        <f>C14+C17</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="45">
-        <f>D14+D17</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="46">
+      <c r="A18" s="103" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="104"/>
+      <c r="C18" s="43">
+        <f>SUM(C15:C17)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="43">
+        <f>SUM(D15:D17)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="44">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="75">
-        <f>F14+F17</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="76">
-        <f>G14+G17</f>
-        <v>0</v>
-      </c>
-      <c r="H18" s="76">
+      <c r="F18" s="65">
+        <f>SUM(F15:F17)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="66">
+        <f>SUM(G15:G17)</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="66">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I18" s="77" t="e">
-        <f>AVERAGE(I14,I17)</f>
+      <c r="I18" s="66" t="e">
+        <f>AVERAGE(I15:I17)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J18" s="77" t="e">
-        <f>AVERAGE(J14,J17)</f>
+      <c r="J18" s="66" t="e">
+        <f>AVERAGE(J15:J17)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="K18" s="78" t="e">
+      <c r="K18" s="67" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L18" s="70">
-        <v>0</v>
-      </c>
-      <c r="M18" s="71">
-        <v>0</v>
-      </c>
-      <c r="N18" s="71">
-        <v>0</v>
-      </c>
-      <c r="O18" s="71">
-        <v>0</v>
-      </c>
-      <c r="P18" s="71">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="71">
-        <v>0</v>
-      </c>
-      <c r="R18" s="71">
-        <v>0</v>
-      </c>
-      <c r="S18" s="71">
-        <v>0</v>
-      </c>
-      <c r="T18" s="72">
-        <v>0</v>
-      </c>
-      <c r="U18" s="73">
-        <v>0</v>
-      </c>
-      <c r="V18" s="71">
-        <v>0</v>
-      </c>
-      <c r="W18" s="71">
-        <v>0</v>
-      </c>
-      <c r="X18" s="71">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="71">
-        <v>0</v>
-      </c>
-      <c r="Z18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AC18" s="74">
-        <v>0</v>
-      </c>
-      <c r="AD18" s="70">
-        <v>0</v>
-      </c>
-      <c r="AE18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AF18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AG18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AH18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AI18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AJ18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AK18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AL18" s="72">
-        <v>0</v>
-      </c>
-      <c r="AM18" s="73">
-        <v>0</v>
-      </c>
-      <c r="AN18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AO18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AP18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AQ18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AR18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AS18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AT18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AU18" s="74">
-        <v>0</v>
-      </c>
-      <c r="AV18" s="70">
-        <v>0</v>
-      </c>
-      <c r="AW18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AX18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AY18" s="71">
-        <v>0</v>
-      </c>
-      <c r="AZ18" s="71">
-        <v>0</v>
-      </c>
-      <c r="BA18" s="71">
-        <v>0</v>
-      </c>
-      <c r="BB18" s="71">
-        <v>0</v>
-      </c>
-      <c r="BC18" s="71">
-        <v>0</v>
-      </c>
-      <c r="BD18" s="74">
+      <c r="L18" s="52">
+        <v>0</v>
+      </c>
+      <c r="M18" s="68">
+        <v>0</v>
+      </c>
+      <c r="N18" s="68">
+        <v>0</v>
+      </c>
+      <c r="O18" s="68">
+        <v>0</v>
+      </c>
+      <c r="P18" s="68">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="68">
+        <v>0</v>
+      </c>
+      <c r="R18" s="68">
+        <v>0</v>
+      </c>
+      <c r="S18" s="68">
+        <v>0</v>
+      </c>
+      <c r="T18" s="69">
+        <v>0</v>
+      </c>
+      <c r="U18" s="54">
+        <v>0</v>
+      </c>
+      <c r="V18" s="68">
+        <v>0</v>
+      </c>
+      <c r="W18" s="68">
+        <v>0</v>
+      </c>
+      <c r="X18" s="68">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="68">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="53">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="52">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AI18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AK18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AL18" s="69">
+        <v>0</v>
+      </c>
+      <c r="AM18" s="54">
+        <v>0</v>
+      </c>
+      <c r="AN18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AO18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AP18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AQ18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AR18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AS18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AT18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AU18" s="53">
+        <v>0</v>
+      </c>
+      <c r="AV18" s="52">
+        <v>0</v>
+      </c>
+      <c r="AW18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AX18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AY18" s="68">
+        <v>0</v>
+      </c>
+      <c r="AZ18" s="68">
+        <v>0</v>
+      </c>
+      <c r="BA18" s="68">
+        <v>0</v>
+      </c>
+      <c r="BB18" s="68">
+        <v>0</v>
+      </c>
+      <c r="BC18" s="68">
+        <v>0</v>
+      </c>
+      <c r="BD18" s="53">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A19" s="103"/>
-      <c r="B19" s="82"/>
-      <c r="C19" s="82"/>
-      <c r="D19" s="82"/>
-      <c r="E19" s="82"/>
-      <c r="F19" s="82"/>
-      <c r="G19" s="82"/>
-      <c r="H19" s="82"/>
-      <c r="I19" s="82"/>
-      <c r="J19" s="82"/>
-      <c r="K19" s="82"/>
-      <c r="L19" s="82"/>
-      <c r="M19" s="82"/>
-      <c r="N19" s="82"/>
-      <c r="O19" s="82"/>
-      <c r="P19" s="82"/>
-      <c r="Q19" s="82"/>
-      <c r="R19" s="82"/>
-      <c r="S19" s="82"/>
-      <c r="T19" s="82"/>
-      <c r="U19" s="1"/>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-      <c r="AA19" s="1"/>
-      <c r="AB19" s="1"/>
-      <c r="AC19" s="1"/>
-      <c r="AD19" s="1"/>
-      <c r="AE19" s="1"/>
-      <c r="AF19" s="1"/>
-      <c r="AG19" s="1"/>
-      <c r="AH19" s="1"/>
-      <c r="AI19" s="1"/>
-      <c r="AJ19" s="1"/>
-      <c r="AK19" s="1"/>
-      <c r="AL19" s="1"/>
-      <c r="AM19" s="1"/>
-      <c r="AN19" s="1"/>
-      <c r="AO19" s="1"/>
-      <c r="AP19" s="1"/>
-      <c r="AQ19" s="1"/>
-      <c r="AR19" s="1"/>
-      <c r="AS19" s="1"/>
-      <c r="AT19" s="1"/>
-      <c r="AU19" s="1"/>
-      <c r="AV19" s="1"/>
-      <c r="AW19" s="1"/>
-      <c r="AX19" s="1"/>
-      <c r="AY19" s="1"/>
-      <c r="AZ19" s="1"/>
-      <c r="BA19" s="1"/>
-      <c r="BB19" s="1"/>
-      <c r="BC19" s="1"/>
-      <c r="BD19" s="1"/>
+      <c r="A19" s="105" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="104"/>
+      <c r="C19" s="45">
+        <f>C14+C18</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="45">
+        <f>D14+D18</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="46">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F19" s="75">
+        <f>F14+F18</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="76">
+        <f>G14+G18</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="76">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="77" t="e">
+        <f>AVERAGE(I14,I18)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="J19" s="77" t="e">
+        <f>AVERAGE(J14,J18)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K19" s="78" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L19" s="70">
+        <v>0</v>
+      </c>
+      <c r="M19" s="71">
+        <v>0</v>
+      </c>
+      <c r="N19" s="71">
+        <v>0</v>
+      </c>
+      <c r="O19" s="71">
+        <v>0</v>
+      </c>
+      <c r="P19" s="71">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="71">
+        <v>0</v>
+      </c>
+      <c r="R19" s="71">
+        <v>0</v>
+      </c>
+      <c r="S19" s="71">
+        <v>0</v>
+      </c>
+      <c r="T19" s="72">
+        <v>0</v>
+      </c>
+      <c r="U19" s="73">
+        <v>0</v>
+      </c>
+      <c r="V19" s="71">
+        <v>0</v>
+      </c>
+      <c r="W19" s="71">
+        <v>0</v>
+      </c>
+      <c r="X19" s="71">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="71">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="74">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="70">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AK19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AL19" s="72">
+        <v>0</v>
+      </c>
+      <c r="AM19" s="73">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AO19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AP19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AQ19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AR19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AS19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AT19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AU19" s="74">
+        <v>0</v>
+      </c>
+      <c r="AV19" s="70">
+        <v>0</v>
+      </c>
+      <c r="AW19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AX19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AY19" s="71">
+        <v>0</v>
+      </c>
+      <c r="AZ19" s="71">
+        <v>0</v>
+      </c>
+      <c r="BA19" s="71">
+        <v>0</v>
+      </c>
+      <c r="BB19" s="71">
+        <v>0</v>
+      </c>
+      <c r="BC19" s="71">
+        <v>0</v>
+      </c>
+      <c r="BD19" s="74">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A20" s="47"/>
-      <c r="B20" s="47"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="47"/>
-      <c r="P20" s="47"/>
-      <c r="Q20" s="47"/>
-      <c r="R20" s="47"/>
-      <c r="S20" s="47"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="13"/>
-      <c r="V20" s="13"/>
+      <c r="A20" s="123"/>
+      <c r="B20" s="87"/>
+      <c r="C20" s="87"/>
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="87"/>
+      <c r="H20" s="87"/>
+      <c r="I20" s="87"/>
+      <c r="J20" s="87"/>
+      <c r="K20" s="87"/>
+      <c r="L20" s="87"/>
+      <c r="M20" s="87"/>
+      <c r="N20" s="87"/>
+      <c r="O20" s="87"/>
+      <c r="P20" s="87"/>
+      <c r="Q20" s="87"/>
+      <c r="R20" s="87"/>
+      <c r="S20" s="87"/>
+      <c r="T20" s="87"/>
+      <c r="U20" s="1"/>
+      <c r="V20" s="1"/>
       <c r="W20" s="1"/>
-      <c r="X20" s="13"/>
-      <c r="Y20" s="13"/>
+      <c r="X20" s="1"/>
+      <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
-      <c r="AA20" s="48"/>
-      <c r="AB20" s="48"/>
-      <c r="AC20" s="48"/>
-      <c r="AD20" s="48"/>
-      <c r="AE20" s="48"/>
-      <c r="AF20" s="48"/>
-      <c r="AG20" s="48"/>
-      <c r="AH20" s="48"/>
-      <c r="AI20" s="48"/>
-      <c r="AJ20" s="48"/>
-      <c r="AK20" s="48"/>
-      <c r="AL20" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="AM20" s="13"/>
-      <c r="AN20" s="13"/>
+      <c r="AA20" s="1"/>
+      <c r="AB20" s="1"/>
+      <c r="AC20" s="1"/>
+      <c r="AD20" s="1"/>
+      <c r="AE20" s="1"/>
+      <c r="AF20" s="1"/>
+      <c r="AG20" s="1"/>
+      <c r="AH20" s="1"/>
+      <c r="AI20" s="1"/>
+      <c r="AJ20" s="1"/>
+      <c r="AK20" s="1"/>
+      <c r="AL20" s="1"/>
+      <c r="AM20" s="1"/>
+      <c r="AN20" s="1"/>
       <c r="AO20" s="1"/>
-      <c r="AP20" s="13"/>
-      <c r="AQ20" s="13"/>
+      <c r="AP20" s="1"/>
+      <c r="AQ20" s="1"/>
       <c r="AR20" s="1"/>
-      <c r="AS20" s="48"/>
-      <c r="AT20" s="48"/>
-      <c r="AU20" s="48"/>
-      <c r="AV20" s="48"/>
-      <c r="AW20" s="48"/>
-      <c r="AX20" s="48"/>
-      <c r="AY20" s="48"/>
-      <c r="AZ20" s="48"/>
-      <c r="BA20" s="48"/>
-      <c r="BB20" s="48"/>
-      <c r="BC20" s="48"/>
-      <c r="BD20" s="3"/>
+      <c r="AS20" s="1"/>
+      <c r="AT20" s="1"/>
+      <c r="AU20" s="1"/>
+      <c r="AV20" s="1"/>
+      <c r="AW20" s="1"/>
+      <c r="AX20" s="1"/>
+      <c r="AY20" s="1"/>
+      <c r="AZ20" s="1"/>
+      <c r="BA20" s="1"/>
+      <c r="BB20" s="1"/>
+      <c r="BC20" s="1"/>
+      <c r="BD20" s="1"/>
     </row>
     <row r="21" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
+      <c r="A21" s="47"/>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="1"/>
-      <c r="U21" s="1"/>
-      <c r="V21" s="1"/>
+      <c r="L21" s="47"/>
+      <c r="M21" s="47"/>
+      <c r="N21" s="47"/>
+      <c r="O21" s="47"/>
+      <c r="P21" s="47"/>
+      <c r="Q21" s="47"/>
+      <c r="R21" s="47"/>
+      <c r="S21" s="47"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="13"/>
+      <c r="V21" s="13"/>
       <c r="W21" s="1"/>
-      <c r="X21" s="1"/>
-      <c r="Y21" s="1"/>
+      <c r="X21" s="13"/>
+      <c r="Y21" s="13"/>
       <c r="Z21" s="1"/>
-      <c r="AA21" s="1"/>
-      <c r="AB21" s="1"/>
-      <c r="AC21" s="1"/>
-      <c r="AD21" s="1"/>
-      <c r="AE21" s="1"/>
-      <c r="AF21" s="1"/>
-      <c r="AG21" s="1"/>
-      <c r="AH21" s="1"/>
-      <c r="AI21" s="1"/>
-      <c r="AJ21" s="1"/>
-      <c r="AK21" s="1"/>
-      <c r="AL21" s="1"/>
-      <c r="AM21" s="1"/>
-      <c r="AN21" s="1"/>
+      <c r="AA21" s="48"/>
+      <c r="AB21" s="48"/>
+      <c r="AC21" s="48"/>
+      <c r="AD21" s="48"/>
+      <c r="AE21" s="48"/>
+      <c r="AF21" s="48"/>
+      <c r="AG21" s="48"/>
+      <c r="AH21" s="48"/>
+      <c r="AI21" s="48"/>
+      <c r="AJ21" s="48"/>
+      <c r="AK21" s="48"/>
+      <c r="AL21" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AM21" s="13"/>
+      <c r="AN21" s="13"/>
       <c r="AO21" s="1"/>
-      <c r="AP21" s="1"/>
-      <c r="AQ21" s="1"/>
+      <c r="AP21" s="13"/>
+      <c r="AQ21" s="13"/>
       <c r="AR21" s="1"/>
-      <c r="AS21" s="1"/>
-      <c r="AT21" s="1"/>
-      <c r="AU21" s="1"/>
-      <c r="AV21" s="1"/>
-      <c r="AW21" s="1"/>
-      <c r="AX21" s="1"/>
-      <c r="AY21" s="1"/>
-      <c r="AZ21" s="1"/>
-      <c r="BA21" s="1"/>
-      <c r="BB21" s="1"/>
-      <c r="BC21" s="1"/>
+      <c r="AS21" s="48"/>
+      <c r="AT21" s="48"/>
+      <c r="AU21" s="48"/>
+      <c r="AV21" s="48"/>
+      <c r="AW21" s="48"/>
+      <c r="AX21" s="48"/>
+      <c r="AY21" s="48"/>
+      <c r="AZ21" s="48"/>
+      <c r="BA21" s="48"/>
+      <c r="BB21" s="48"/>
+      <c r="BC21" s="48"/>
       <c r="BD21" s="3"/>
     </row>
     <row r="22" spans="1:56" ht="16.5" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="49"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
-      <c r="T22" s="13"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="1"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
-      <c r="AA22" s="102"/>
-      <c r="AB22" s="82"/>
-      <c r="AC22" s="82"/>
-      <c r="AD22" s="82"/>
-      <c r="AE22" s="82"/>
-      <c r="AF22" s="82"/>
-      <c r="AG22" s="82"/>
-      <c r="AH22" s="82"/>
-      <c r="AI22" s="82"/>
-      <c r="AJ22" s="82"/>
-      <c r="AK22" s="82"/>
-      <c r="AL22" s="13"/>
+      <c r="AA22" s="1"/>
+      <c r="AB22" s="1"/>
+      <c r="AC22" s="1"/>
+      <c r="AD22" s="1"/>
+      <c r="AE22" s="1"/>
+      <c r="AF22" s="1"/>
+      <c r="AG22" s="1"/>
+      <c r="AH22" s="1"/>
+      <c r="AI22" s="1"/>
+      <c r="AJ22" s="1"/>
+      <c r="AK22" s="1"/>
+      <c r="AL22" s="1"/>
       <c r="AM22" s="1"/>
       <c r="AN22" s="1"/>
       <c r="AO22" s="1"/>
       <c r="AP22" s="1"/>
       <c r="AQ22" s="1"/>
       <c r="AR22" s="1"/>
-      <c r="AS22" s="86"/>
-      <c r="AT22" s="87"/>
-      <c r="AU22" s="87"/>
-      <c r="AV22" s="87"/>
-      <c r="AW22" s="87"/>
-      <c r="AX22" s="87"/>
-      <c r="AY22" s="87"/>
-      <c r="AZ22" s="87"/>
-      <c r="BA22" s="87"/>
-      <c r="BB22" s="87"/>
-      <c r="BC22" s="87"/>
-      <c r="BD22" s="1"/>
+      <c r="AS22" s="1"/>
+      <c r="AT22" s="1"/>
+      <c r="AU22" s="1"/>
+      <c r="AV22" s="1"/>
+      <c r="AW22" s="1"/>
+      <c r="AX22" s="1"/>
+      <c r="AY22" s="1"/>
+      <c r="AZ22" s="1"/>
+      <c r="BA22" s="1"/>
+      <c r="BB22" s="1"/>
+      <c r="BC22" s="1"/>
+      <c r="BD22" s="3"/>
     </row>
     <row r="23" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
+      <c r="A23" s="1"/>
+      <c r="B23" s="49"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
@@ -3836,106 +3981,102 @@
       <c r="X23" s="1"/>
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
-      <c r="AA23" s="3"/>
-      <c r="AB23" s="3"/>
-      <c r="AC23" s="3"/>
-      <c r="AD23" s="3"/>
-      <c r="AE23" s="3"/>
-      <c r="AF23" s="3"/>
-      <c r="AG23" s="3"/>
-      <c r="AH23" s="3"/>
-      <c r="AI23" s="3"/>
-      <c r="AJ23" s="3"/>
-      <c r="AK23" s="1"/>
+      <c r="AA23" s="122"/>
+      <c r="AB23" s="87"/>
+      <c r="AC23" s="87"/>
+      <c r="AD23" s="87"/>
+      <c r="AE23" s="87"/>
+      <c r="AF23" s="87"/>
+      <c r="AG23" s="87"/>
+      <c r="AH23" s="87"/>
+      <c r="AI23" s="87"/>
+      <c r="AJ23" s="87"/>
+      <c r="AK23" s="87"/>
       <c r="AL23" s="13"/>
       <c r="AM23" s="1"/>
       <c r="AN23" s="1"/>
       <c r="AO23" s="1"/>
       <c r="AP23" s="1"/>
-      <c r="AQ23" s="94" t="s">
+      <c r="AQ23" s="1"/>
+      <c r="AR23" s="1"/>
+      <c r="AS23" s="121"/>
+      <c r="AT23" s="119"/>
+      <c r="AU23" s="119"/>
+      <c r="AV23" s="119"/>
+      <c r="AW23" s="119"/>
+      <c r="AX23" s="119"/>
+      <c r="AY23" s="119"/>
+      <c r="AZ23" s="119"/>
+      <c r="BA23" s="119"/>
+      <c r="BB23" s="119"/>
+      <c r="BC23" s="119"/>
+      <c r="BD23" s="1"/>
+    </row>
+    <row r="24" spans="1:56" ht="16.5" customHeight="1">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="13"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="13"/>
+      <c r="T24" s="13"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="1"/>
+      <c r="W24" s="1"/>
+      <c r="X24" s="1"/>
+      <c r="Y24" s="1"/>
+      <c r="Z24" s="1"/>
+      <c r="AA24" s="3"/>
+      <c r="AB24" s="3"/>
+      <c r="AC24" s="3"/>
+      <c r="AD24" s="3"/>
+      <c r="AE24" s="3"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="3"/>
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="3"/>
+      <c r="AJ24" s="3"/>
+      <c r="AK24" s="1"/>
+      <c r="AL24" s="13"/>
+      <c r="AM24" s="1"/>
+      <c r="AN24" s="1"/>
+      <c r="AO24" s="1"/>
+      <c r="AP24" s="1"/>
+      <c r="AQ24" s="110" t="s">
         <v>37</v>
       </c>
-      <c r="AR23" s="82"/>
-      <c r="AS23" s="82"/>
-      <c r="AT23" s="82"/>
-      <c r="AU23" s="82"/>
-      <c r="AV23" s="82"/>
-      <c r="AW23" s="82"/>
-      <c r="AX23" s="82"/>
-      <c r="AY23" s="82"/>
-      <c r="AZ23" s="82"/>
-      <c r="BA23" s="82"/>
-      <c r="BB23" s="82"/>
-      <c r="BC23" s="82"/>
-      <c r="BD23" s="82"/>
-    </row>
-    <row r="24" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A24" s="50" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="47"/>
-      <c r="M24" s="47"/>
-      <c r="N24" s="95" t="s">
-        <v>16</v>
-      </c>
-      <c r="O24" s="82"/>
-      <c r="P24" s="82"/>
-      <c r="Q24" s="82"/>
-      <c r="R24" s="82"/>
-      <c r="S24" s="82"/>
-      <c r="T24" s="82"/>
-      <c r="U24" s="82"/>
-      <c r="V24" s="82"/>
-      <c r="W24" s="82"/>
-      <c r="X24" s="82"/>
-      <c r="Y24" s="82"/>
-      <c r="Z24" s="82"/>
-      <c r="AA24" s="82"/>
-      <c r="AB24" s="82"/>
-      <c r="AC24" s="82"/>
-      <c r="AD24" s="82"/>
-      <c r="AE24" s="82"/>
-      <c r="AF24" s="82"/>
-      <c r="AG24" s="82"/>
-      <c r="AH24" s="82"/>
-      <c r="AI24" s="82"/>
-      <c r="AJ24" s="47"/>
-      <c r="AK24" s="47"/>
-      <c r="AL24" s="47"/>
-      <c r="AM24" s="47"/>
-      <c r="AN24" s="47"/>
-      <c r="AO24" s="47"/>
-      <c r="AP24" s="47"/>
-      <c r="AQ24" s="47"/>
-      <c r="AR24" s="47"/>
-      <c r="AS24" s="47"/>
-      <c r="AT24" s="47"/>
-      <c r="AU24" s="47"/>
-      <c r="AV24" s="47"/>
-      <c r="AW24" s="47"/>
-      <c r="AX24" s="47"/>
-      <c r="AY24" s="47"/>
-      <c r="AZ24" s="47"/>
-      <c r="BA24" s="47"/>
-      <c r="BB24" s="47"/>
-      <c r="BC24" s="47"/>
-      <c r="BD24" s="47"/>
+      <c r="AR24" s="87"/>
+      <c r="AS24" s="87"/>
+      <c r="AT24" s="87"/>
+      <c r="AU24" s="87"/>
+      <c r="AV24" s="87"/>
+      <c r="AW24" s="87"/>
+      <c r="AX24" s="87"/>
+      <c r="AY24" s="87"/>
+      <c r="AZ24" s="87"/>
+      <c r="BA24" s="87"/>
+      <c r="BB24" s="87"/>
+      <c r="BC24" s="87"/>
+      <c r="BD24" s="87"/>
     </row>
     <row r="25" spans="1:56" ht="16.5" customHeight="1">
       <c r="A25" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" s="47"/>
+        <v>15</v>
+      </c>
+      <c r="B25" s="51"/>
       <c r="C25" s="47"/>
       <c r="D25" s="47"/>
       <c r="E25" s="47"/>
@@ -3947,28 +4088,30 @@
       <c r="K25" s="1"/>
       <c r="L25" s="47"/>
       <c r="M25" s="47"/>
-      <c r="N25" s="82"/>
-      <c r="O25" s="82"/>
-      <c r="P25" s="82"/>
-      <c r="Q25" s="82"/>
-      <c r="R25" s="82"/>
-      <c r="S25" s="82"/>
-      <c r="T25" s="82"/>
-      <c r="U25" s="82"/>
-      <c r="V25" s="82"/>
-      <c r="W25" s="82"/>
-      <c r="X25" s="82"/>
-      <c r="Y25" s="82"/>
-      <c r="Z25" s="82"/>
-      <c r="AA25" s="82"/>
-      <c r="AB25" s="82"/>
-      <c r="AC25" s="82"/>
-      <c r="AD25" s="82"/>
-      <c r="AE25" s="82"/>
-      <c r="AF25" s="82"/>
-      <c r="AG25" s="82"/>
-      <c r="AH25" s="82"/>
-      <c r="AI25" s="82"/>
+      <c r="N25" s="111" t="s">
+        <v>16</v>
+      </c>
+      <c r="O25" s="87"/>
+      <c r="P25" s="87"/>
+      <c r="Q25" s="87"/>
+      <c r="R25" s="87"/>
+      <c r="S25" s="87"/>
+      <c r="T25" s="87"/>
+      <c r="U25" s="87"/>
+      <c r="V25" s="87"/>
+      <c r="W25" s="87"/>
+      <c r="X25" s="87"/>
+      <c r="Y25" s="87"/>
+      <c r="Z25" s="87"/>
+      <c r="AA25" s="87"/>
+      <c r="AB25" s="87"/>
+      <c r="AC25" s="87"/>
+      <c r="AD25" s="87"/>
+      <c r="AE25" s="87"/>
+      <c r="AF25" s="87"/>
+      <c r="AG25" s="87"/>
+      <c r="AH25" s="87"/>
+      <c r="AI25" s="87"/>
       <c r="AJ25" s="47"/>
       <c r="AK25" s="47"/>
       <c r="AL25" s="47"/>
@@ -3993,7 +4136,7 @@
     </row>
     <row r="26" spans="1:56" ht="16.5" customHeight="1">
       <c r="A26" s="50" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B26" s="47"/>
       <c r="C26" s="47"/>
@@ -4007,46 +4150,44 @@
       <c r="K26" s="1"/>
       <c r="L26" s="47"/>
       <c r="M26" s="47"/>
-      <c r="N26" s="82"/>
-      <c r="O26" s="82"/>
-      <c r="P26" s="82"/>
-      <c r="Q26" s="82"/>
-      <c r="R26" s="82"/>
-      <c r="S26" s="82"/>
-      <c r="T26" s="82"/>
-      <c r="U26" s="82"/>
-      <c r="V26" s="82"/>
-      <c r="W26" s="82"/>
-      <c r="X26" s="82"/>
-      <c r="Y26" s="82"/>
-      <c r="Z26" s="82"/>
-      <c r="AA26" s="82"/>
-      <c r="AB26" s="82"/>
-      <c r="AC26" s="82"/>
-      <c r="AD26" s="82"/>
-      <c r="AE26" s="82"/>
-      <c r="AF26" s="82"/>
-      <c r="AG26" s="82"/>
-      <c r="AH26" s="82"/>
-      <c r="AI26" s="82"/>
+      <c r="N26" s="87"/>
+      <c r="O26" s="87"/>
+      <c r="P26" s="87"/>
+      <c r="Q26" s="87"/>
+      <c r="R26" s="87"/>
+      <c r="S26" s="87"/>
+      <c r="T26" s="87"/>
+      <c r="U26" s="87"/>
+      <c r="V26" s="87"/>
+      <c r="W26" s="87"/>
+      <c r="X26" s="87"/>
+      <c r="Y26" s="87"/>
+      <c r="Z26" s="87"/>
+      <c r="AA26" s="87"/>
+      <c r="AB26" s="87"/>
+      <c r="AC26" s="87"/>
+      <c r="AD26" s="87"/>
+      <c r="AE26" s="87"/>
+      <c r="AF26" s="87"/>
+      <c r="AG26" s="87"/>
+      <c r="AH26" s="87"/>
+      <c r="AI26" s="87"/>
       <c r="AJ26" s="47"/>
       <c r="AK26" s="47"/>
       <c r="AL26" s="47"/>
       <c r="AM26" s="47"/>
-      <c r="AN26" s="92" t="s">
-        <v>17</v>
-      </c>
-      <c r="AO26" s="82"/>
-      <c r="AP26" s="82"/>
-      <c r="AQ26" s="82"/>
-      <c r="AR26" s="82"/>
-      <c r="AS26" s="82"/>
-      <c r="AT26" s="82"/>
-      <c r="AU26" s="82"/>
-      <c r="AV26" s="82"/>
-      <c r="AW26" s="82"/>
-      <c r="AX26" s="82"/>
-      <c r="AY26" s="82"/>
+      <c r="AN26" s="47"/>
+      <c r="AO26" s="47"/>
+      <c r="AP26" s="47"/>
+      <c r="AQ26" s="47"/>
+      <c r="AR26" s="47"/>
+      <c r="AS26" s="47"/>
+      <c r="AT26" s="47"/>
+      <c r="AU26" s="47"/>
+      <c r="AV26" s="47"/>
+      <c r="AW26" s="47"/>
+      <c r="AX26" s="47"/>
+      <c r="AY26" s="47"/>
       <c r="AZ26" s="47"/>
       <c r="BA26" s="47"/>
       <c r="BB26" s="47"/>
@@ -4055,7 +4196,7 @@
     </row>
     <row r="27" spans="1:56" ht="16.5" customHeight="1">
       <c r="A27" s="50" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B27" s="47"/>
       <c r="C27" s="47"/>
@@ -4069,46 +4210,46 @@
       <c r="K27" s="1"/>
       <c r="L27" s="47"/>
       <c r="M27" s="47"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="82"/>
-      <c r="P27" s="82"/>
-      <c r="Q27" s="82"/>
-      <c r="R27" s="82"/>
-      <c r="S27" s="82"/>
-      <c r="T27" s="82"/>
-      <c r="U27" s="82"/>
-      <c r="V27" s="82"/>
-      <c r="W27" s="82"/>
-      <c r="X27" s="82"/>
-      <c r="Y27" s="82"/>
-      <c r="Z27" s="82"/>
-      <c r="AA27" s="82"/>
-      <c r="AB27" s="82"/>
-      <c r="AC27" s="82"/>
-      <c r="AD27" s="82"/>
-      <c r="AE27" s="82"/>
-      <c r="AF27" s="82"/>
-      <c r="AG27" s="82"/>
-      <c r="AH27" s="82"/>
-      <c r="AI27" s="82"/>
+      <c r="N27" s="87"/>
+      <c r="O27" s="87"/>
+      <c r="P27" s="87"/>
+      <c r="Q27" s="87"/>
+      <c r="R27" s="87"/>
+      <c r="S27" s="87"/>
+      <c r="T27" s="87"/>
+      <c r="U27" s="87"/>
+      <c r="V27" s="87"/>
+      <c r="W27" s="87"/>
+      <c r="X27" s="87"/>
+      <c r="Y27" s="87"/>
+      <c r="Z27" s="87"/>
+      <c r="AA27" s="87"/>
+      <c r="AB27" s="87"/>
+      <c r="AC27" s="87"/>
+      <c r="AD27" s="87"/>
+      <c r="AE27" s="87"/>
+      <c r="AF27" s="87"/>
+      <c r="AG27" s="87"/>
+      <c r="AH27" s="87"/>
+      <c r="AI27" s="87"/>
       <c r="AJ27" s="47"/>
       <c r="AK27" s="47"/>
       <c r="AL27" s="47"/>
       <c r="AM27" s="47"/>
-      <c r="AN27" s="93" t="s">
-        <v>20</v>
-      </c>
-      <c r="AO27" s="82"/>
-      <c r="AP27" s="82"/>
-      <c r="AQ27" s="82"/>
-      <c r="AR27" s="82"/>
-      <c r="AS27" s="82"/>
-      <c r="AT27" s="82"/>
-      <c r="AU27" s="82"/>
-      <c r="AV27" s="82"/>
-      <c r="AW27" s="82"/>
-      <c r="AX27" s="82"/>
-      <c r="AY27" s="82"/>
+      <c r="AN27" s="112" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO27" s="87"/>
+      <c r="AP27" s="87"/>
+      <c r="AQ27" s="87"/>
+      <c r="AR27" s="87"/>
+      <c r="AS27" s="87"/>
+      <c r="AT27" s="87"/>
+      <c r="AU27" s="87"/>
+      <c r="AV27" s="87"/>
+      <c r="AW27" s="87"/>
+      <c r="AX27" s="87"/>
+      <c r="AY27" s="87"/>
       <c r="AZ27" s="47"/>
       <c r="BA27" s="47"/>
       <c r="BB27" s="47"/>
@@ -4116,62 +4257,66 @@
       <c r="BD27" s="47"/>
     </row>
     <row r="28" spans="1:56" ht="16.5" customHeight="1">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
+      <c r="A28" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="47"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="82"/>
-      <c r="O28" s="82"/>
-      <c r="P28" s="82"/>
-      <c r="Q28" s="82"/>
-      <c r="R28" s="82"/>
-      <c r="S28" s="82"/>
-      <c r="T28" s="82"/>
-      <c r="U28" s="82"/>
-      <c r="V28" s="82"/>
-      <c r="W28" s="82"/>
-      <c r="X28" s="82"/>
-      <c r="Y28" s="82"/>
-      <c r="Z28" s="82"/>
-      <c r="AA28" s="82"/>
-      <c r="AB28" s="82"/>
-      <c r="AC28" s="82"/>
-      <c r="AD28" s="82"/>
-      <c r="AE28" s="82"/>
-      <c r="AF28" s="82"/>
-      <c r="AG28" s="82"/>
-      <c r="AH28" s="82"/>
-      <c r="AI28" s="82"/>
-      <c r="AJ28" s="1"/>
-      <c r="AK28" s="1"/>
-      <c r="AL28" s="1"/>
-      <c r="AM28" s="1"/>
-      <c r="AN28" s="1"/>
-      <c r="AO28" s="1"/>
-      <c r="AP28" s="1"/>
-      <c r="AQ28" s="1"/>
-      <c r="AR28" s="1"/>
-      <c r="AS28" s="1"/>
-      <c r="AT28" s="1"/>
-      <c r="AU28" s="1"/>
-      <c r="AV28" s="1"/>
-      <c r="AW28" s="1"/>
-      <c r="AX28" s="1"/>
-      <c r="AY28" s="1"/>
-      <c r="AZ28" s="1"/>
-      <c r="BA28" s="1"/>
-      <c r="BB28" s="1"/>
-      <c r="BC28" s="1"/>
-      <c r="BD28" s="1"/>
+      <c r="L28" s="47"/>
+      <c r="M28" s="47"/>
+      <c r="N28" s="87"/>
+      <c r="O28" s="87"/>
+      <c r="P28" s="87"/>
+      <c r="Q28" s="87"/>
+      <c r="R28" s="87"/>
+      <c r="S28" s="87"/>
+      <c r="T28" s="87"/>
+      <c r="U28" s="87"/>
+      <c r="V28" s="87"/>
+      <c r="W28" s="87"/>
+      <c r="X28" s="87"/>
+      <c r="Y28" s="87"/>
+      <c r="Z28" s="87"/>
+      <c r="AA28" s="87"/>
+      <c r="AB28" s="87"/>
+      <c r="AC28" s="87"/>
+      <c r="AD28" s="87"/>
+      <c r="AE28" s="87"/>
+      <c r="AF28" s="87"/>
+      <c r="AG28" s="87"/>
+      <c r="AH28" s="87"/>
+      <c r="AI28" s="87"/>
+      <c r="AJ28" s="47"/>
+      <c r="AK28" s="47"/>
+      <c r="AL28" s="47"/>
+      <c r="AM28" s="47"/>
+      <c r="AN28" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="AO28" s="87"/>
+      <c r="AP28" s="87"/>
+      <c r="AQ28" s="87"/>
+      <c r="AR28" s="87"/>
+      <c r="AS28" s="87"/>
+      <c r="AT28" s="87"/>
+      <c r="AU28" s="87"/>
+      <c r="AV28" s="87"/>
+      <c r="AW28" s="87"/>
+      <c r="AX28" s="87"/>
+      <c r="AY28" s="87"/>
+      <c r="AZ28" s="47"/>
+      <c r="BA28" s="47"/>
+      <c r="BB28" s="47"/>
+      <c r="BC28" s="47"/>
+      <c r="BD28" s="47"/>
     </row>
     <row r="29" spans="1:56" ht="16.5" customHeight="1">
       <c r="A29" s="1"/>
@@ -4187,28 +4332,28 @@
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
-      <c r="U29" s="1"/>
-      <c r="V29" s="1"/>
-      <c r="W29" s="1"/>
-      <c r="X29" s="1"/>
-      <c r="Y29" s="1"/>
-      <c r="Z29" s="1"/>
-      <c r="AA29" s="1"/>
-      <c r="AB29" s="1"/>
-      <c r="AC29" s="1"/>
-      <c r="AD29" s="1"/>
-      <c r="AE29" s="1"/>
-      <c r="AF29" s="1"/>
-      <c r="AG29" s="1"/>
-      <c r="AH29" s="1"/>
-      <c r="AI29" s="1"/>
+      <c r="N29" s="87"/>
+      <c r="O29" s="87"/>
+      <c r="P29" s="87"/>
+      <c r="Q29" s="87"/>
+      <c r="R29" s="87"/>
+      <c r="S29" s="87"/>
+      <c r="T29" s="87"/>
+      <c r="U29" s="87"/>
+      <c r="V29" s="87"/>
+      <c r="W29" s="87"/>
+      <c r="X29" s="87"/>
+      <c r="Y29" s="87"/>
+      <c r="Z29" s="87"/>
+      <c r="AA29" s="87"/>
+      <c r="AB29" s="87"/>
+      <c r="AC29" s="87"/>
+      <c r="AD29" s="87"/>
+      <c r="AE29" s="87"/>
+      <c r="AF29" s="87"/>
+      <c r="AG29" s="87"/>
+      <c r="AH29" s="87"/>
+      <c r="AI29" s="87"/>
       <c r="AJ29" s="1"/>
       <c r="AK29" s="1"/>
       <c r="AL29" s="1"/>
@@ -15715,19 +15860,91 @@
       <c r="BC227" s="1"/>
       <c r="BD227" s="1"/>
     </row>
+    <row r="228" spans="1:56" ht="16.5" customHeight="1">
+      <c r="A228" s="1"/>
+      <c r="B228" s="1"/>
+      <c r="C228" s="1"/>
+      <c r="D228" s="1"/>
+      <c r="E228" s="1"/>
+      <c r="F228" s="1"/>
+      <c r="G228" s="1"/>
+      <c r="H228" s="1"/>
+      <c r="I228" s="1"/>
+      <c r="J228" s="1"/>
+      <c r="K228" s="1"/>
+      <c r="L228" s="1"/>
+      <c r="M228" s="1"/>
+      <c r="N228" s="1"/>
+      <c r="O228" s="1"/>
+      <c r="P228" s="1"/>
+      <c r="Q228" s="1"/>
+      <c r="R228" s="1"/>
+      <c r="S228" s="1"/>
+      <c r="T228" s="1"/>
+      <c r="U228" s="1"/>
+      <c r="V228" s="1"/>
+      <c r="W228" s="1"/>
+      <c r="X228" s="1"/>
+      <c r="Y228" s="1"/>
+      <c r="Z228" s="1"/>
+      <c r="AA228" s="1"/>
+      <c r="AB228" s="1"/>
+      <c r="AC228" s="1"/>
+      <c r="AD228" s="1"/>
+      <c r="AE228" s="1"/>
+      <c r="AF228" s="1"/>
+      <c r="AG228" s="1"/>
+      <c r="AH228" s="1"/>
+      <c r="AI228" s="1"/>
+      <c r="AJ228" s="1"/>
+      <c r="AK228" s="1"/>
+      <c r="AL228" s="1"/>
+      <c r="AM228" s="1"/>
+      <c r="AN228" s="1"/>
+      <c r="AO228" s="1"/>
+      <c r="AP228" s="1"/>
+      <c r="AQ228" s="1"/>
+      <c r="AR228" s="1"/>
+      <c r="AS228" s="1"/>
+      <c r="AT228" s="1"/>
+      <c r="AU228" s="1"/>
+      <c r="AV228" s="1"/>
+      <c r="AW228" s="1"/>
+      <c r="AX228" s="1"/>
+      <c r="AY228" s="1"/>
+      <c r="AZ228" s="1"/>
+      <c r="BA228" s="1"/>
+      <c r="BB228" s="1"/>
+      <c r="BC228" s="1"/>
+      <c r="BD228" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="AY10:BA10"/>
-    <mergeCell ref="BB10:BD10"/>
-    <mergeCell ref="AJ10:AL10"/>
-    <mergeCell ref="U10:W10"/>
-    <mergeCell ref="AM10:AO10"/>
-    <mergeCell ref="AP10:AR10"/>
-    <mergeCell ref="AS4:AU4"/>
-    <mergeCell ref="P4:X4"/>
-    <mergeCell ref="Y4:AB4"/>
-    <mergeCell ref="AC4:AO4"/>
-    <mergeCell ref="AP4:AR4"/>
+    <mergeCell ref="AQ24:BD24"/>
+    <mergeCell ref="N25:AI29"/>
+    <mergeCell ref="AN27:AY27"/>
+    <mergeCell ref="AN28:AY28"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="C9:E10"/>
+    <mergeCell ref="R10:T10"/>
+    <mergeCell ref="AS23:BC23"/>
+    <mergeCell ref="AA23:AK23"/>
+    <mergeCell ref="A20:T20"/>
+    <mergeCell ref="AF6:AO6"/>
+    <mergeCell ref="AQ6:AV6"/>
+    <mergeCell ref="AW6:BD6"/>
+    <mergeCell ref="X10:Z10"/>
+    <mergeCell ref="AA10:AC10"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="K6:O6"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="L9:T9"/>
     <mergeCell ref="A1:BD2"/>
     <mergeCell ref="A3:BD3"/>
     <mergeCell ref="P6:U6"/>
@@ -15744,31 +15961,17 @@
     <mergeCell ref="AD9:AL9"/>
     <mergeCell ref="AV9:BD9"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="K6:O6"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="C4:L4"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="M4:O4"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="L9:T9"/>
-    <mergeCell ref="AQ23:BD23"/>
-    <mergeCell ref="N24:AI28"/>
-    <mergeCell ref="AN26:AY26"/>
-    <mergeCell ref="AN27:AY27"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="C9:E10"/>
-    <mergeCell ref="R10:T10"/>
-    <mergeCell ref="AS22:BC22"/>
-    <mergeCell ref="AA22:AK22"/>
-    <mergeCell ref="A19:T19"/>
-    <mergeCell ref="AF6:AO6"/>
-    <mergeCell ref="AQ6:AV6"/>
-    <mergeCell ref="AW6:BD6"/>
-    <mergeCell ref="X10:Z10"/>
-    <mergeCell ref="AA10:AC10"/>
+    <mergeCell ref="AS4:AU4"/>
+    <mergeCell ref="P4:X4"/>
+    <mergeCell ref="Y4:AB4"/>
+    <mergeCell ref="AC4:AO4"/>
+    <mergeCell ref="AP4:AR4"/>
+    <mergeCell ref="AY10:BA10"/>
+    <mergeCell ref="BB10:BD10"/>
+    <mergeCell ref="AJ10:AL10"/>
+    <mergeCell ref="U10:W10"/>
+    <mergeCell ref="AM10:AO10"/>
+    <mergeCell ref="AP10:AR10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup scale="68" orientation="landscape" r:id="rId1"/>

</xml_diff>